<commit_message>
Add ACGME duty-hour audit; eliminate 7-day work streaks; disambiguate names
- New dutyhours.py audits the schedule against ACGME limits: <=80h/wk averaged
  over 4 weeks (busiest 72.8h), no duty period >28h (max 24h), and >=1 day off
  per week. All pass.
- Smoothing pass removes every 7-consecutive-workday run (max streak now 6) by
  handing that week's Thursday day-off to the affected outside rotator (an LSH
  covers the Thursday short call); one Monday runs a single short call. Kennedy
  is never pulled in.
- Grid now shows a first initial after each surname (AHLUWALIA Sr vs AHLUWALIA Sa,
  SAEED U vs SAEED S, etc.) so the two Ahluwalias and two Saeeds are distinct.
- RULES_COMPLIANCE.md gains a duty-hour section; workbooks regenerated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J6EM8SxuZs5C898HeFBgt7
</commit_message>
<xml_diff>
--- a/intern_schedule_2026-2027/schedules/TYP_April_2027.xlsx
+++ b/intern_schedule_2026-2027/schedules/TYP_April_2027.xlsx
@@ -517,17 +517,17 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI</t>
+          <t>ZAIDI H</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>RIVERA</t>
+          <t>RIVERA A</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>ALMADHOOB</t>
+          <t>ALMADHOOB M</t>
         </is>
       </c>
     </row>
@@ -542,17 +542,17 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>OGHENESUME</t>
+          <t>OGHENESUME O</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI, RIVERA</t>
+          <t>ZAIDI H, RIVERA A</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>ALMADHOOB</t>
+          <t>ALMADHOOB M</t>
         </is>
       </c>
     </row>
@@ -567,13 +567,13 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>RIVERA</t>
+          <t>RIVERA A</t>
         </is>
       </c>
       <c r="D5" s="4" t="n"/>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>RIVERA  (24H)</t>
+          <t>RIVERA A  (24H)</t>
         </is>
       </c>
     </row>
@@ -588,13 +588,13 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>ALMADHOOB</t>
+          <t>ALMADHOOB M</t>
         </is>
       </c>
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>ZAIDI</t>
+          <t>ZAIDI H</t>
         </is>
       </c>
     </row>
@@ -609,17 +609,17 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>OGHENESUME</t>
+          <t>OGHENESUME O</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>RIVERA, ALMADHOOB</t>
+          <t>RIVERA A, ALMADHOOB M</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI</t>
+          <t>ZAIDI H</t>
         </is>
       </c>
     </row>
@@ -634,17 +634,17 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>RIVERA</t>
+          <t>RIVERA A</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>OGHENESUME, ALMADHOOB</t>
+          <t>OGHENESUME O, ALMADHOOB M</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI</t>
+          <t>ZAIDI H</t>
         </is>
       </c>
     </row>
@@ -659,17 +659,17 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>ALMADHOOB</t>
+          <t>ALMADHOOB M</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>OGHENESUME, RIVERA</t>
+          <t>OGHENESUME O, RIVERA A</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI</t>
+          <t>ZAIDI H</t>
         </is>
       </c>
     </row>
@@ -684,17 +684,17 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>RIVERA</t>
+          <t>RIVERA A</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>ALMADHOOB</t>
+          <t>OGHENESUME O</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI</t>
+          <t>ZAIDI H</t>
         </is>
       </c>
     </row>
@@ -709,17 +709,17 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>OGHENESUME</t>
+          <t>OGHENESUME O</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>RIVERA, ALMADHOOB</t>
+          <t>RIVERA A, ALMADHOOB M</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI</t>
+          <t>ZAIDI H</t>
         </is>
       </c>
     </row>
@@ -734,13 +734,13 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>ALMADHOOB</t>
+          <t>ALMADHOOB M</t>
         </is>
       </c>
       <c r="D12" s="4" t="n"/>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>ALMADHOOB  (24H)</t>
+          <t>ALMADHOOB M  (24H)</t>
         </is>
       </c>
     </row>
@@ -755,13 +755,13 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>RIVERA</t>
+          <t>RIVERA A</t>
         </is>
       </c>
       <c r="D13" s="5" t="n"/>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>OGHENESUME</t>
+          <t>OGHENESUME O</t>
         </is>
       </c>
     </row>
@@ -776,17 +776,17 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI</t>
+          <t>ZAIDI H</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>RIVERA, ALMADHOOB</t>
+          <t>RIVERA A, ALMADHOOB M</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>OGHENESUME</t>
+          <t>OGHENESUME O</t>
         </is>
       </c>
     </row>
@@ -801,17 +801,17 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>ALMADHOOB</t>
+          <t>ALMADHOOB M</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI, RIVERA</t>
+          <t>ZAIDI H, RIVERA A</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>OGHENESUME</t>
+          <t>OGHENESUME O</t>
         </is>
       </c>
     </row>
@@ -826,17 +826,17 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>RIVERA</t>
+          <t>RIVERA A</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI, ALMADHOOB</t>
+          <t>ZAIDI H, ALMADHOOB M</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>OGHENESUME</t>
+          <t>OGHENESUME O</t>
         </is>
       </c>
     </row>
@@ -851,17 +851,17 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>ALMADHOOB</t>
+          <t>ALMADHOOB M</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>RIVERA</t>
+          <t>RIVERA A</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>OGHENESUME</t>
+          <t>OGHENESUME O</t>
         </is>
       </c>
     </row>
@@ -876,17 +876,17 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>RIVERA</t>
+          <t>RIVERA A</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI, ALMADHOOB</t>
+          <t>ZAIDI H, ALMADHOOB M</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>OGHENESUME</t>
+          <t>OGHENESUME O</t>
         </is>
       </c>
     </row>
@@ -901,13 +901,13 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>ZAIDI</t>
+          <t>ZAIDI H</t>
         </is>
       </c>
       <c r="D19" s="4" t="n"/>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>ZAIDI  (24H)</t>
+          <t>ZAIDI H  (24H)</t>
         </is>
       </c>
     </row>
@@ -922,13 +922,13 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>ALMADHOOB</t>
+          <t>ALMADHOOB M</t>
         </is>
       </c>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>RIVERA</t>
+          <t>RIVERA A</t>
         </is>
       </c>
     </row>
@@ -943,17 +943,17 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>OGHENESUME</t>
+          <t>OGHENESUME O</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI, AHLUWALIA</t>
+          <t>ZAIDI H, AHLUWALIA Sa</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>RIVERA</t>
+          <t>RIVERA A</t>
         </is>
       </c>
     </row>
@@ -968,17 +968,17 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>AHLUWALIA</t>
+          <t>AHLUWALIA Sa</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI, OGHENESUME</t>
+          <t>ZAIDI H, OGHENESUME O</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>RIVERA</t>
+          <t>RIVERA A</t>
         </is>
       </c>
     </row>
@@ -993,17 +993,17 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI</t>
+          <t>ZAIDI H</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>OGHENESUME, AHLUWALIA</t>
+          <t>OGHENESUME O, AHLUWALIA Sa</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>RIVERA</t>
+          <t>RIVERA A</t>
         </is>
       </c>
     </row>
@@ -1018,17 +1018,17 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>AHLUWALIA</t>
+          <t>AHLUWALIA Sa</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI</t>
+          <t>ZAIDI H</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>RIVERA</t>
+          <t>RIVERA A</t>
         </is>
       </c>
     </row>
@@ -1043,17 +1043,17 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI</t>
+          <t>ZAIDI H</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>OGHENESUME, AHLUWALIA</t>
+          <t>OGHENESUME O, AHLUWALIA Sa</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>RIVERA</t>
+          <t>RIVERA A</t>
         </is>
       </c>
     </row>
@@ -1068,13 +1068,13 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>OGHENESUME</t>
+          <t>OGHENESUME O</t>
         </is>
       </c>
       <c r="D26" s="4" t="n"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>OGHENESUME  (24H)</t>
+          <t>OGHENESUME O  (24H)</t>
         </is>
       </c>
     </row>
@@ -1089,13 +1089,13 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>RIVERA</t>
+          <t>RIVERA A</t>
         </is>
       </c>
       <c r="D27" s="5" t="n"/>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>AHLUWALIA</t>
+          <t>AHLUWALIA Sa</t>
         </is>
       </c>
     </row>
@@ -1110,17 +1110,17 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI</t>
+          <t>ZAIDI H</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>OGHENESUME, GABALLAH</t>
+          <t>OGHENESUME O, GABALLAH B</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>AHLUWALIA</t>
+          <t>AHLUWALIA Sa</t>
         </is>
       </c>
     </row>
@@ -1135,17 +1135,17 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>GABALLAH</t>
+          <t>GABALLAH B</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI, OGHENESUME</t>
+          <t>ZAIDI H, OGHENESUME O</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>AHLUWALIA</t>
+          <t>AHLUWALIA Sa</t>
         </is>
       </c>
     </row>
@@ -1160,17 +1160,17 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>OGHENESUME</t>
+          <t>OGHENESUME O</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI, GABALLAH</t>
+          <t>ZAIDI H, GABALLAH B</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>AHLUWALIA</t>
+          <t>AHLUWALIA Sa</t>
         </is>
       </c>
     </row>
@@ -1185,17 +1185,17 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>GABALLAH</t>
+          <t>GABALLAH B</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>OGHENESUME</t>
+          <t>OGHENESUME O</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>AHLUWALIA</t>
+          <t>AHLUWALIA Sa</t>
         </is>
       </c>
     </row>
@@ -1210,17 +1210,17 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>ZAIDI</t>
+          <t>ZAIDI H</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>OGHENESUME, GABALLAH</t>
+          <t>OGHENESUME O, GABALLAH B</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>AHLUWALIA</t>
+          <t>AHLUWALIA Sa</t>
         </is>
       </c>
     </row>

</xml_diff>